<commit_message>
Update Dallas Open projections
</commit_message>
<xml_diff>
--- a/draws/dallas2026.xlsx
+++ b/draws/dallas2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cadecarlson/EDACCloud/tf-site/draws/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA580889-6FBA-DD4F-866C-28FA6AC17101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EDE9A0-B6BB-674B-B6C5-4430ABDE53FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Draw" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>DrawPosition</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>dallas-2026</t>
+  </si>
+  <si>
+    <t>2026-02-09</t>
+  </si>
+  <si>
+    <t>2026-02-15</t>
   </si>
 </sst>
 </file>
@@ -200,7 +206,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -805,16 +811,16 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4">
-        <v>46062</v>
+      <c r="B6" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4">
-        <v>46068</v>
+      <c r="B7" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>